<commit_message>
Aula 12 trabalho com Excel e CRUD dentro dele.
</commit_message>
<xml_diff>
--- a/aula12/cadastro_alunos.xlsx
+++ b/aula12/cadastro_alunos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,106 +436,121 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ddd</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>gggg</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.9</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>llll</t>
+          <t>Bernardo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gggg</t>
+          <t>34</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>uuuu</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>oooo</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.9</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>wwww</t>
+          <t>Micael</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>rrrr</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>iiii</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>rrrr</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>yyyy</t>
+          <t>aaa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ffff</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8.300000000000001</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8.9</v>
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>6.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>